<commit_message>
docs(week7): consolidate changes 1-6 and architecture into one PR; regenerate exports
Supersedes the stacked PRs #197-#203. The live ruleset dismisses approvals
on every push and squash-merging a stack forces a rebase push after each
merge, so seven serial re-approvals become one.

- #198 (change 2) cherry-picked onto the stack tip; its STATE entry merged
  as the union.
- Exports regenerated against the full set: CONNECTSPHERE BACKLOGS CAA
  031026.xlsx (56 Release 1 stories, 78 product), PROJECT TEST CASES CAA
  031026.xlsx (311 cases) and the legacy copy, docs/testing/tc-coverage.md.
- docs/source-of-truth.md: BDR export row moved here from #194 so the two
  PRs share no file.
- .agents/STATE.md and .agents/JOURNAL.md: entries moved here from #194,
  #195, #196 and #204 for the same reason, plus one entry for this
  consolidation and the live strict=false ruleset change.
</commit_message>
<xml_diff>
--- a/docs/CONNECTSPHERE BACKLOGS CAA 031026.xlsx
+++ b/docs/CONNECTSPHERE BACKLOGS CAA 031026.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1889,30 +1889,89 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>E05 Venue Catalogue &amp; Availability</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>E05-S06</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Mark a venue temporarily unavailable over existing bookings</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>As a Venue Staff member, I want to mark a venue temporarily unavailable for maintenance, equipment failure, renovation, a safety concern or another operational reason, even when events are already booked in it, so that affected bookings are identified and their Coordinators can arrange an alternative without the events themselves being cancelled.
+New story from the Week 7 Customer Changes (C-66). It supersedes E05-S04 Scenario 2, which refused a block over a confirmed booking; E05-S04 is in the Sprint 2 sprint backlog and is not edited (T-67, T-74). Estimate to be set by planning poker at Sprint 3 planning (T-73). Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Scenario 1 - Unavailability recorded with a reason
+Given I am viewing a venue When I mark it unavailable for a period and choose a reason category from maintenance, equipment failure, renovation, safety concern or other, with a free-text note Then the unavailability is saved with the period, the category, the note and my identity, and the calendar shows the period as Blocked
+Scenario 2 - Overlapping bookings become Conflicting, not released
+Given the venue has a Pending request and a Confirmed booking inside the period When I save the unavailability Then the save succeeds, both bookings are marked Conflicting, neither is released or cancelled, and the two affected events are listed to me on save
+Scenario 3 - The event itself is untouched
+Given a Confirmed event's booking has just become Conflicting When anyone views that event Then its status is still Confirmed, every other arrangement is intact, and a venue-conflict flag with the reason category is shown; the event changes status only when its Coordinator acts (assumes O-24)
+Scenario 4 - Affected Coordinators informed
+Given the unavailability made one or more bookings Conflicting When it is saved Then the Coordinator of each affected event receives an in-app and email notification naming the venue, the period, the reason category and the event, and stating that alternative arrangements are required (assumes O-25)
+Scenario 5 - End date required and extendable
+Given I am recording an unavailability When I omit the end date and time Then the save is refused; and Given a saved unavailability When I extend its end Then bookings newly inside the longer period are handled as in Scenario 2 (assumes O-23)
+Scenario 6 - Unavailability shortened or ended early
+Given a booking is Conflicting only because of an unavailability When I shorten or end that unavailability so the booking no longer overlaps it Then the Conflicting flag clears and the booking stands as it was; a booking the Coordinator has already cancelled or replaced is not restored (assumes O-26)
+Checklist
+- Mark a venue unavailable for a period with a reason category and a note, including when Pending or Confirmed bookings fall inside the period
+- See the affected events listed on save and their bookings marked Conflicting, with none released or cancelled
+- Confirm the affected events keep their status and other arrangements, with a visible venue-conflict flag
+- Confirm each affected Coordinator is notified in-app and by email
+- Be refused an unavailability with no end date and time
+- Confirm shortening or ending an unavailability clears the Conflicting flag on bookings it no longer touches
+- Confirm E05-S04's existing block, shorten and remove behaviour still works for periods with no bookings</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>C-66, C-48, C-61, T-28, T-67, T-74, O-23, O-24, O-25, O-26</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>E06 Venue Search &amp; Booking</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>E06-S01</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Search for suitable venues</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to search venues by date, time, attendance, capacity, layout, accessibility and facilities so that I can shortlist options for an event quickly.</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Matching venues listed
 Given venues exist that match all my criteria and are available When I run the search Then those venues are listed with their capacity, layouts and facilities
@@ -1933,43 +1992,43 @@
 - Apply several filters together in one search</t>
         </is>
       </c>
-      <c r="G27" s="2" t="n">
+      <c r="G28" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>B-08, C-65, T-66</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>E06 Venue Search &amp; Booking</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>E06-S02</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Check venue suitability against event requirements</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want the system to compare a venue against the event's recorded requirements so that I do not request a venue that cannot meet them.</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Suitability shown for the event
 Given an event has recorded requirements When I view a venue in the context of the event Then a suitability status is shown for the event
@@ -1987,43 +2046,43 @@
 - Confirm suitability is advisory and does not itself block a booking request</t>
         </is>
       </c>
-      <c r="G28" s="2" t="n">
+      <c r="G29" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>C-06, T-13, T-21, B-08</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>E06 Venue Search &amp; Booking</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>E06-S03</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Request a venue booking</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to submit a venue booking request for an event so that Venue Staff can review it and decide whether the venue can be provided.</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Request created as Pending
 Given an event has recorded requirements and no pending request When I submit a booking request for a venue Then the request is created with status Pending, the venue calendar shows the period as Tentative, and the Venue Staff are notified
@@ -2051,43 +2110,43 @@
 - View the status of each of my booking requests</t>
         </is>
       </c>
-      <c r="G29" s="2" t="n">
+      <c r="G30" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>C-01, C-16, C-17, C-37, C-46, C-60, T-20, T-49, C-65, T-66, C-67, T-68, O-27, O-29, O-30</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>E06 Venue Search &amp; Booking</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>E06-S04</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Decide on a venue booking request</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>As a Venue Staff member, I want to approve or reject booking requests and record my reasoning so that Coordinators receive a clear, traceable decision.</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Request approved and confirmed
 Given a booking request is pending and the venue is free for the period When I approve it Then the booking becomes Confirmed, the venue calendar is updated and the Coordinator is notified
@@ -2107,44 +2166,44 @@
 - Confirm the Coordinator is notified of either decision</t>
         </is>
       </c>
-      <c r="G30" s="2" t="n">
+      <c r="G31" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>C-08, T-39, C-65, T-66</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>E06 Venue Search &amp; Booking</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>E06-S05</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Hold a venue tentatively</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to place a tentative hold on a venue so that it is not taken by another event while the arrangements are still being finalised, and I want the hold to expire at a known time so that venues are not reserved indefinitely.
 The expiry scenarios come from the Week 7 Customer Changes (C-68, T-69) and reverse the earlier position that no expiry was required (C-01, C-16, C-60, T-49). Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Tentative hold placed
 Given a venue is free for the period When I place a tentative hold Then the calendar shows the period as Tentative, the hold is recorded against my event, and the hold carries an expiry date and time set to 48 hours from creation by default, which Venue Staff may change on the hold (assumes O-31)
@@ -2177,43 +2236,43 @@
 - Confirm Venue Staff can extend an unexpired hold and the extension is logged (assumes O-34)</t>
         </is>
       </c>
-      <c r="G31" s="2" t="n">
+      <c r="G32" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>C-01, C-16, C-37, C-60, T-49, C-65, T-66, C-68, T-69, O-31, O-32, O-33, O-34</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>E06 Venue Search &amp; Booking</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>E06-S06</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Prevent double-booking of a venue</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>As a Venue Staff member, I want to be blocked from approving a booking that overlaps an existing confirmed booking for the same venue so that a venue is never committed to two events at once.</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Overlapping approval blocked
 Given a venue has a confirmed booking When I attempt to approve another request overlapping that period Then approval is blocked and the conflicting booking is identified
@@ -2234,43 +2293,43 @@
 - Confirm no venue ever holds two confirmed bookings over the same period</t>
         </is>
       </c>
-      <c r="G32" s="2" t="n">
+      <c r="G33" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>C-46, T-22, C-65, T-66, C-67, T-68</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>E07 Equipment &amp; Technical Support</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>E07-S01</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Maintain the equipment catalogue</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>As a Technical Support Staff member, I want to maintain equipment records including type, quantity, location and operational status so that availability checks are based on accurate data.</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Item added and reservable
 Given I am adding an equipment item When I save its type, description, quantity, location and operational status Then it becomes available for reservation
@@ -2287,43 +2346,43 @@
 - Confirm retired items no longer appear in availability checks</t>
         </is>
       </c>
-      <c r="G33" s="2" t="n">
+      <c r="G34" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>E07 Equipment &amp; Technical Support</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>E07-S02</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Request equipment for an event</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to record the equipment an event needs, with quantities, so that Technical Support Staff can check whether it can be provided.</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Equipment recorded against an event
 Given I am planning an approved event When I add equipment items with quantities to an event Then the request is saved against the event and the Technical Support Staff are notified
@@ -2339,43 +2398,43 @@
 - Amend or remove an equipment request before it is reserved</t>
         </is>
       </c>
-      <c r="G34" s="2" t="n">
+      <c r="G35" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>T-25</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>E07 Equipment &amp; Technical Support</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>E07-S03</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Check equipment availability</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>As a Technical Support Staff member, I want to see how much of an item is free for a given date and time so that I can decide whether a request can be met.</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Reserved and faulty stock excluded
 Given some items are reserved for other events in the period When I check availability Then the free quantity excludes those reservations and any items marked damaged or under maintenance
@@ -2391,43 +2450,43 @@
 - Confirm the same item can serve two events at non-overlapping times</t>
         </is>
       </c>
-      <c r="G35" s="2" t="n">
+      <c r="G36" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>C-07, C-20</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>E07 Equipment &amp; Technical Support</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>E07-S04</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>Reserve equipment for an event</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>As a Technical Support Staff member, I want to reserve equipment for an event so that limited equipment is not committed to two events at the same time.</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Full reservation recorded
 Given sufficient equipment is free for the period When I reserve the requested quantity Then the reservation is recorded against the event and the Event Coordinator is notified
@@ -2446,43 +2505,43 @@
 - Receive confirmation showing the event, date, time, item and quantity</t>
         </is>
       </c>
-      <c r="G36" s="2" t="n">
+      <c r="G37" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>C-21, T-24, B-09</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>E07 Equipment &amp; Technical Support</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>E07-S05</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>Mark equipment as unavailable</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>As a Technical Support Staff member, I want to mark equipment as damaged or under maintenance so that it is not treated as available for events.</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Item marked unavailable
 Given an item has no reservations in the period When I mark it unavailable with a reason and a period Then it is excluded from availability checks for that period
@@ -2495,43 +2554,43 @@
 - Return an item to service, restoring it to availability checks</t>
         </is>
       </c>
-      <c r="G37" s="2" t="n">
+      <c r="G38" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>B-04</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>E07 Equipment &amp; Technical Support</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>E07-S06</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Request technical support for an event</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to request on-site technical support for an event and describe what is needed so that suitable staff can be allocated.</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Support request recorded
 Given an event requires technical support When I submit a request describing the support and the times it is needed Then the Technical Support Staff are notified and the request is recorded against the event
@@ -2547,43 +2606,43 @@
 - Mark an event as requiring no technical support</t>
         </is>
       </c>
-      <c r="G38" s="2" t="n">
+      <c r="G39" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>C-22, T-23</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>E07 Equipment &amp; Technical Support</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>E07-S07</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Assign and manage technical staff for an event</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>As a Technical Support Staff member, I want to assign and manage available colleagues to support an event so that the right people are on site at the right time.</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Available colleague assigned
 Given an event has an open technical support request and a colleague is available for its times When I assign them Then they are notified and the assignment appears on their schedule
@@ -2602,44 +2661,44 @@
 - Confirm the staff member is notified when assigned or removed</t>
         </is>
       </c>
-      <c r="G39" s="2" t="n">
+      <c r="G40" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>C-39</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>E08 Readiness &amp; Confirmation</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>E08-S03</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Confirm an event</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to confirm an event once the event's arrangements are complete so that the Event Organiser and Attendees can rely on the details.
 Amended in place for the Week 7 Customer Changes (C-70, T-71; this story is To Do, T-74). Completing the arrangements no longer sets Confirmed directly: it lets the Coordinator submit the event for its Operational Safety Check, which moves it to the new Safety Review status, and the Safety Officer's approval (E08-S06) is what sets Confirmed. The readiness checks below are unchanged in substance; what they now gate is the submission. Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - All arrangements complete, event submitted for safety review
 Given every venue booking on the event is Confirmed or has been withdrawn, at least one is Confirmed, its full requested equipment is reserved and any requested technical support is assigned When I submit the event for its Operational Safety Check Then the status becomes Safety Review, the Safety Officer is notified, the Organiser is told the event is awaiting its safety check, and the event becomes Confirmed only when the Safety Officer approves it (E08-S06) (C-67, T-68, C-70, T-71; assumes O-28, O-39, O-40)
@@ -2665,43 +2724,43 @@
 - Confirm the Event Organiser is notified with the full confirmed details</t>
         </is>
       </c>
-      <c r="G40" s="2" t="n">
+      <c r="G41" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>C-13, C-39, C-59, C-63, T-02, T-24, T-27, C-67, T-68, O-28, C-70, T-71, T-74, O-39, O-40</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>E08 Readiness &amp; Confirmation</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>E08-S04</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>Revert a confirmed event to planning</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to return a confirmed event to planning when an arrangement breaks so that its status reflects reality.</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Reverted with a recorded reason
 Given an event is Confirmed When I revert it to Planning and record a reason Then the status becomes Planning and the Event Organiser is notified with the reason
@@ -2720,43 +2779,43 @@
 - Confirm a reverted event must pass the Operational Safety Check again before it is Confirmed again</t>
         </is>
       </c>
-      <c r="G41" s="2" t="n">
+      <c r="G42" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>C-48, T-03, T-28, C-70, T-71</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="I42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>E08 Readiness &amp; Confirmation</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>E08-S05</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>Complete an event</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want an event to become Completed once it has taken place so that attendance can be recorded and the event closed.</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Auto-completed after the end time
 Given an event is Confirmed and its end time has passed When the system next evaluates it Then the status becomes Completed
@@ -2774,44 +2833,44 @@
 - Confirm the transition is recorded in the activity log</t>
         </is>
       </c>
-      <c r="G42" s="2" t="n">
+      <c r="G43" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>T-03, T-26, T-48</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="I43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>E08 Readiness &amp; Confirmation</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>E08-S06</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>Conduct the Operational Safety Check as the Safety Officer</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>As a Safety Officer, I want to review the operational safety of each event whose venue and technical arrangements are confirmed, and approve it, reject its safety arrangement or request changes, so that no event proceeds to preparation until it is safe to run.
 New story from the Week 7 Customer Changes (C-70) and the seventh role (T-72). The Safety Review status it works on sits between Planning and Confirmed as an interim placement (T-71); O-39 asks the customer to confirm. The customer guarantees a response, so there is no timeout path. Estimate at Sprint 3 planning (T-73). Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Events awaiting review listed with what the check needs
 Given events are in Safety Review When I open my queue Then each shows the event name, date and time, every confirmed venue with its capacity, layout and known restrictions, expected attendance, accessibility requirements, equipment and its placement, and the time it entered Safety Review, oldest first
@@ -2844,41 +2903,41 @@
 - Confirm every decision is in the activity log</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr"/>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>C-70, T-71, T-72, T-73, T-74, O-39, O-40, O-41, O-42, O-43</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>E09 Attendee Registration</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>E09-S01</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>Register for an event</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>As an Attendee, I want to register for a confirmed event so that my place is reserved and I receive the event information.</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Place reserved in an open event
 Given an event is Confirmed, registration is open and places remain When I submit the required registration information Then my place is reserved and I receive a confirmation containing the event details
@@ -2899,43 +2958,43 @@
 - Be refused registration for an event that is not Confirmed</t>
         </is>
       </c>
-      <c r="G44" s="2" t="n">
+      <c r="G45" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>C-35, T-48, C-67, T-68, O-30</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>E09 Attendee Registration</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>E09-S02</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>Enforce registration capacity</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>As an Event Organiser, I want registration to stop at the booked venue's capacity so that more people do not register than the venue can hold.</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Venue capacity enforced
 Given the event's capacity is the booked venue's capacity When registrations reach that number Then further registrations are refused
@@ -2956,43 +3015,43 @@
 - Confirm a manual addition is distinguishable from a normal registration</t>
         </is>
       </c>
-      <c r="G45" s="2" t="n">
+      <c r="G46" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>C-05, C-58, T-30, T-31, T-50, B-11</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>E09 Attendee Registration</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>E09-S03</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>Control the registration period</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>As an Event Organiser, I want to set when registration opens and closes, and when withdrawal closes, so that Attendees can act only during the permitted windows.</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Before registration opens
 Given the registration opening date has not been reached When an Attendee views the event Then registration is shown as not yet open and the opening date is stated
@@ -3011,43 +3070,43 @@
 - Be warned when setting a closing date after the event has started</t>
         </is>
       </c>
-      <c r="G46" s="2" t="n">
+      <c r="G47" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>C-24, C-44, T-42</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>E09 Attendee Registration</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>E09-S04</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>Join the waiting list</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>As an Attendee, I want to join the waiting list when an event is full so that I can still attend if a place is released.</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Joined a full event's list
 Given an event is full and the waiting list is enabled When I join the waiting list Then I am added and told I will be notified when a place is released
@@ -3066,43 +3125,43 @@
 - Confirm no waiting list is offered when the Organiser has disabled it</t>
         </is>
       </c>
-      <c r="G47" s="2" t="n">
+      <c r="G48" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>C-23, T-33, T-46, B-10</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>E09 Attendee Registration</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>E09-S05</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>Withdraw my registration</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>As an Attendee, I want to withdraw my registration so that my place is released to someone else.</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Registration withdrawn
 Given I am registered and the withdrawal deadline has not passed When I withdraw Then my registration is cancelled and the place becomes available again
@@ -3114,43 +3173,43 @@
 - Be refused after the withdrawal deadline, with a contact provided</t>
         </is>
       </c>
-      <c r="G48" s="2" t="n">
+      <c r="G49" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>C-24, T-48, B-10</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>E09 Attendee Registration</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>E09-S06</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Record attendance</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to record which registered Attendees actually attended the event so that registration and attendance can be distinguished.</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Attendance marked after completion
 Given an event has status Completed When I mark an Attendee as attended for an event Then their record shows attended and the registration figure is unchanged
@@ -3166,43 +3225,43 @@
 - View registration and attendance counts side by side for the event</t>
         </is>
       </c>
-      <c r="G49" s="2" t="n">
+      <c r="G50" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>C-45</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>E09 Attendee Registration</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>E09-S07</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>View registrations for my event</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>As an Event Organiser, I want to view the list of Attendees registered for my event so that I can plan for the numbers attending the event.</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Registrations grouped by event
 Given Attendees have registered for my event When I open its registration list Then I see each Attendee's name, email address and contact number
@@ -3220,43 +3279,43 @@
 - Be refused access to registration lists for events I do not manage</t>
         </is>
       </c>
-      <c r="G50" s="2" t="n">
+      <c r="G51" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>C-26, T-32, O-05</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="I51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>E10 Changes, Rescheduling &amp; Cancellation</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>E10-S01</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>Request a change after submission</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>As an Event Organiser, I want to request a change to my event after it has been submitted or confirmed so that the arrangements reflect what I now need.</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Change request recorded
 Given my event has been approved or confirmed When I submit a change request describing what should change Then the assigned Coordinator is notified and the request is recorded against the event
@@ -3275,43 +3334,43 @@
 - Be notified when the Coordinator approves or declines the request</t>
         </is>
       </c>
-      <c r="G51" s="2" t="n">
+      <c r="G52" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>C-14, C-52, C-54, T-16</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="I52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>E10 Changes, Rescheduling &amp; Cancellation</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>E10-S02</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>Distinguish minor edits from arrangement-affecting changes</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want the system to tell me when a change affects arrangements already confirmed so that I re-check them rather than assuming they still hold.</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Attendance beyond capacity flagged
 Given an event has one or more confirmed venue bookings When its expected attendance is increased Then each venue booking whose governing headcount (the booking's own headcount where set, otherwise the event's attendance) now exceeds that venue's capacity is flagged for review, and the others are not (C-67; assumes O-27) and the Venue Staff are notified
@@ -3332,43 +3391,43 @@
 - Confirm affected Venue Staff and Technical Support Staff are notified</t>
         </is>
       </c>
-      <c r="G52" s="2" t="n">
+      <c r="G53" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="I53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>E10 Changes, Rescheduling &amp; Cancellation</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>E10-S04</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>Cancel an event</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to cancel an event and release its arrangements so that venues and equipment do not stay committed to something that will not happen.</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Event cancelled, arrangements released
 Given an Event Organiser requests cancellation When I cancel the event and record a reason Then its status becomes Cancelled, its venue booking and equipment reservations are released, the venue calendar is updated and the affected staff are notified
@@ -3387,43 +3446,98 @@
 - Confirm a cancelled event is read-only and shows its reason and date</t>
         </is>
       </c>
-      <c r="G53" s="2" t="n">
+      <c r="G54" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>C-14, C-54, T-07, T-48</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="I54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>E10 Changes, Rescheduling &amp; Cancellation</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>E10-S05</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Handle a venue lost from a confirmed event</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>As an Event Coordinator, I want to be alerted when a venue becomes unavailable for one of my events and to find and request a replacement from the event itself, so that I can arrange an alternative before Attendees are affected while the original event information is preserved.
+Returned to Release 1 by the Week 7 Customer Changes (C-66, T-67). The three-point estimate is carried from the original backlog and re-estimated at Sprint 3 planning (T-73). The alert itself is raised by E05-S06; this story is what the Coordinator does with it. Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Scenario 1 - Lost venue flags the event
+Given my event has a Pending or Confirmed venue booking When Venue Staff mark that venue unavailable over the booking's period (E05-S06) Then I am notified, the booking shows as Conflicting on the event, and the event is flagged as needing alternative arrangements while its status and every other arrangement stay as they were (assumes O-24)
+Scenario 2 - Flagged event offers a replacement search
+Given my event is flagged When I open it Then the reason category, the period and the affected booking are shown, the original venue, dates and requirements are preserved, and I can start a venue search (E06-S01) for the same event from that screen
+Scenario 3 - Replacement requested without losing the original
+Given I have found a replacement venue When I submit a booking request for it (E06-S03) Then the request is created for the same event alongside the Conflicting booking, and I may cancel the Conflicting booking explicitly once the replacement is Confirmed; nothing is cancelled for me
+Scenario 4 - Organiser and Attendees told on the actual change
+Given I confirm a replacement venue When the venue of a Confirmed event changes Then the Organiser and registered Attendees are notified of the new venue through the existing venue-change routing (E11-S01), and not earlier (assumes O-25)
+Checklist
+- Be notified when a venue I have booked is marked unavailable over my booking
+- See the reason, period and affected booking on the event, with the original event information intact
+- Start a venue search for the same event from the flagged event
+- Request a replacement venue while the Conflicting booking remains on the event until I cancel it
+- Confirm the Organiser and registered Attendees are told of the venue change only when it actually happens</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>C-66, C-61, T-28, T-67, T-73, T-74, O-24, O-25</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>E11 Notifications &amp; Reminders</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>E11-S01</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>Notify users about events they are involved in</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>As a user involved in an event, I want to be notified when its status or arrangements change so that I do not have to keep checking the system and nobody continues working from outdated information.</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Status change notified
 Given I am a recipient under the approved routing matrix When an event status changes or a booking decision is made Then I receive a notification stating what changed, when, and which event it concerns, unless I performed the action myself
@@ -3451,43 +3565,43 @@
 - Mark a notification as read</t>
         </is>
       </c>
-      <c r="G54" s="2" t="n">
+      <c r="G56" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>C-04, C-29, C-53, T-35, T-36, T-44, T-48, T-64, C-68, T-69, O-33, C-69, T-70, C-70, T-71</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="I56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>E14 Audit &amp; History</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>E14-S02</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>Record significant actions in an activity log</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>As a ConnectSphere staff member, I want significant actions to be recorded so that we can determine who did what and when.</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Status change recorded
 Given an event status changes When the change completes Then an entry is recorded with the actor, the action, the affected event and the time
@@ -3507,15 +3621,15 @@
 - Confirm log entries cannot be edited or deleted by any user</t>
         </is>
       </c>
-      <c r="G55" s="2" t="n">
+      <c r="G57" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>T-04</t>
         </is>
       </c>
-      <c r="I55" s="2" t="inlineStr">
+      <c r="I57" s="2" t="inlineStr">
         <is>
           <t>Le Xin</t>
         </is>
@@ -3532,7 +3646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I78"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5240,25 +5354,80 @@
       <c r="A36" s="2" t="inlineStr"/>
       <c r="B36" s="2" t="inlineStr">
         <is>
+          <t>E05 Venue Catalogue &amp; Availability</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>E05-S06</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Mark a venue temporarily unavailable over existing bookings</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>As a Venue Staff member, I want to mark a venue temporarily unavailable for maintenance, equipment failure, renovation, a safety concern or another operational reason, even when events are already booked in it, so that affected bookings are identified and their Coordinators can arrange an alternative without the events themselves being cancelled.
+New story from the Week 7 Customer Changes (C-66). It supersedes E05-S04 Scenario 2, which refused a block over a confirmed booking; E05-S04 is in the Sprint 2 sprint backlog and is not edited (T-67, T-74). Estimate to be set by planning poker at Sprint 3 planning (T-73). Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Scenario 1 - Unavailability recorded with a reason
+Given I am viewing a venue When I mark it unavailable for a period and choose a reason category from maintenance, equipment failure, renovation, safety concern or other, with a free-text note Then the unavailability is saved with the period, the category, the note and my identity, and the calendar shows the period as Blocked
+Scenario 2 - Overlapping bookings become Conflicting, not released
+Given the venue has a Pending request and a Confirmed booking inside the period When I save the unavailability Then the save succeeds, both bookings are marked Conflicting, neither is released or cancelled, and the two affected events are listed to me on save
+Scenario 3 - The event itself is untouched
+Given a Confirmed event's booking has just become Conflicting When anyone views that event Then its status is still Confirmed, every other arrangement is intact, and a venue-conflict flag with the reason category is shown; the event changes status only when its Coordinator acts (assumes O-24)
+Scenario 4 - Affected Coordinators informed
+Given the unavailability made one or more bookings Conflicting When it is saved Then the Coordinator of each affected event receives an in-app and email notification naming the venue, the period, the reason category and the event, and stating that alternative arrangements are required (assumes O-25)
+Scenario 5 - End date required and extendable
+Given I am recording an unavailability When I omit the end date and time Then the save is refused; and Given a saved unavailability When I extend its end Then bookings newly inside the longer period are handled as in Scenario 2 (assumes O-23)
+Scenario 6 - Unavailability shortened or ended early
+Given a booking is Conflicting only because of an unavailability When I shorten or end that unavailability so the booking no longer overlaps it Then the Conflicting flag clears and the booking stands as it was; a booking the Coordinator has already cancelled or replaced is not restored (assumes O-26)
+Checklist
+- Mark a venue unavailable for a period with a reason category and a note, including when Pending or Confirmed bookings fall inside the period
+- See the affected events listed on save and their bookings marked Conflicting, with none released or cancelled
+- Confirm the affected events keep their status and other arrangements, with a visible venue-conflict flag
+- Confirm each affected Coordinator is notified in-app and by email
+- Be refused an unavailability with no end date and time
+- Confirm shortening or ending an unavailability clears the Conflicting flag on bookings it no longer touches
+- Confirm E05-S04's existing block, shorten and remove behaviour still works for periods with no bookings</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>C-66, C-48, C-61, T-28, T-67, T-74, O-23, O-24, O-25, O-26</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr"/>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
           <t>E06 Venue Search &amp; Booking</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>E06-S01</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>Search for suitable venues</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to search venues by date, time, attendance, capacity, layout, accessibility and facilities so that I can shortlist options for an event quickly.</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Matching venues listed
 Given venues exist that match all my criteria and are available When I run the search Then those venues are listed with their capacity, layouts and facilities
@@ -5279,39 +5448,39 @@
 - Apply several filters together in one search</t>
         </is>
       </c>
-      <c r="G36" s="2" t="n">
+      <c r="G37" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>B-08, C-65, T-66</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr"/>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr"/>
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>E06 Venue Search &amp; Booking</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>E06-S02</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>Check venue suitability against event requirements</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want the system to compare a venue against the event's recorded requirements so that I do not request a venue that cannot meet them.</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Suitability shown for the event
 Given an event has recorded requirements When I view a venue in the context of the event Then a suitability status is shown for the event
@@ -5329,39 +5498,39 @@
 - Confirm suitability is advisory and does not itself block a booking request</t>
         </is>
       </c>
-      <c r="G37" s="2" t="n">
+      <c r="G38" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>C-06, T-13, T-21, B-08</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr"/>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr"/>
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>E06 Venue Search &amp; Booking</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>E06-S03</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Request a venue booking</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to submit a venue booking request for an event so that Venue Staff can review it and decide whether the venue can be provided.</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Request created as Pending
 Given an event has recorded requirements and no pending request When I submit a booking request for a venue Then the request is created with status Pending, the venue calendar shows the period as Tentative, and the Venue Staff are notified
@@ -5389,39 +5558,39 @@
 - View the status of each of my booking requests</t>
         </is>
       </c>
-      <c r="G38" s="2" t="n">
+      <c r="G39" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>C-01, C-16, C-17, C-37, C-46, C-60, T-20, T-49, C-65, T-66, C-67, T-68, O-27, O-29, O-30</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr"/>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr"/>
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>E06 Venue Search &amp; Booking</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>E06-S04</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Decide on a venue booking request</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>As a Venue Staff member, I want to approve or reject booking requests and record my reasoning so that Coordinators receive a clear, traceable decision.</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Request approved and confirmed
 Given a booking request is pending and the venue is free for the period When I approve it Then the booking becomes Confirmed, the venue calendar is updated and the Coordinator is notified
@@ -5441,40 +5610,40 @@
 - Confirm the Coordinator is notified of either decision</t>
         </is>
       </c>
-      <c r="G39" s="2" t="n">
+      <c r="G40" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>C-08, T-39, C-65, T-66</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr"/>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr"/>
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>E06 Venue Search &amp; Booking</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>E06-S05</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Hold a venue tentatively</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to place a tentative hold on a venue so that it is not taken by another event while the arrangements are still being finalised, and I want the hold to expire at a known time so that venues are not reserved indefinitely.
 The expiry scenarios come from the Week 7 Customer Changes (C-68, T-69) and reverse the earlier position that no expiry was required (C-01, C-16, C-60, T-49). Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Tentative hold placed
 Given a venue is free for the period When I place a tentative hold Then the calendar shows the period as Tentative, the hold is recorded against my event, and the hold carries an expiry date and time set to 48 hours from creation by default, which Venue Staff may change on the hold (assumes O-31)
@@ -5507,39 +5676,39 @@
 - Confirm Venue Staff can extend an unexpired hold and the extension is logged (assumes O-34)</t>
         </is>
       </c>
-      <c r="G40" s="2" t="n">
+      <c r="G41" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>C-01, C-16, C-37, C-60, T-49, C-65, T-66, C-68, T-69, O-31, O-32, O-33, O-34</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr"/>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr"/>
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>E06 Venue Search &amp; Booking</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>E06-S06</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>Prevent double-booking of a venue</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>As a Venue Staff member, I want to be blocked from approving a booking that overlaps an existing confirmed booking for the same venue so that a venue is never committed to two events at once.</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Overlapping approval blocked
 Given a venue has a confirmed booking When I attempt to approve another request overlapping that period Then approval is blocked and the conflicting booking is identified
@@ -5560,39 +5729,39 @@
 - Confirm no venue ever holds two confirmed bookings over the same period</t>
         </is>
       </c>
-      <c r="G41" s="2" t="n">
+      <c r="G42" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>C-46, T-22, C-65, T-66, C-67, T-68</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr"/>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="I42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr"/>
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>E07 Equipment &amp; Technical Support</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>E07-S01</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>Maintain the equipment catalogue</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>As a Technical Support Staff member, I want to maintain equipment records including type, quantity, location and operational status so that availability checks are based on accurate data.</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Item added and reservable
 Given I am adding an equipment item When I save its type, description, quantity, location and operational status Then it becomes available for reservation
@@ -5609,39 +5778,39 @@
 - Confirm retired items no longer appear in availability checks</t>
         </is>
       </c>
-      <c r="G42" s="2" t="n">
+      <c r="G43" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr"/>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="I43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr"/>
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>E07 Equipment &amp; Technical Support</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>E07-S02</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>Request equipment for an event</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to record the equipment an event needs, with quantities, so that Technical Support Staff can check whether it can be provided.</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Equipment recorded against an event
 Given I am planning an approved event When I add equipment items with quantities to an event Then the request is saved against the event and the Technical Support Staff are notified
@@ -5657,39 +5826,39 @@
 - Amend or remove an equipment request before it is reserved</t>
         </is>
       </c>
-      <c r="G43" s="2" t="n">
+      <c r="G44" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>T-25</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr"/>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr"/>
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>E07 Equipment &amp; Technical Support</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>E07-S03</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>Check equipment availability</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>As a Technical Support Staff member, I want to see how much of an item is free for a given date and time so that I can decide whether a request can be met.</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Reserved and faulty stock excluded
 Given some items are reserved for other events in the period When I check availability Then the free quantity excludes those reservations and any items marked damaged or under maintenance
@@ -5705,39 +5874,39 @@
 - Confirm the same item can serve two events at non-overlapping times</t>
         </is>
       </c>
-      <c r="G44" s="2" t="n">
+      <c r="G45" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>C-07, C-20</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr"/>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr"/>
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>E07 Equipment &amp; Technical Support</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>E07-S04</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>Reserve equipment for an event</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>As a Technical Support Staff member, I want to reserve equipment for an event so that limited equipment is not committed to two events at the same time.</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Full reservation recorded
 Given sufficient equipment is free for the period When I reserve the requested quantity Then the reservation is recorded against the event and the Event Coordinator is notified
@@ -5756,39 +5925,39 @@
 - Receive confirmation showing the event, date, time, item and quantity</t>
         </is>
       </c>
-      <c r="G45" s="2" t="n">
+      <c r="G46" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>C-21, T-24, B-09</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr"/>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr"/>
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>E07 Equipment &amp; Technical Support</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>E07-S05</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>Mark equipment as unavailable</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>As a Technical Support Staff member, I want to mark equipment as damaged or under maintenance so that it is not treated as available for events.</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Item marked unavailable
 Given an item has no reservations in the period When I mark it unavailable with a reason and a period Then it is excluded from availability checks for that period
@@ -5801,39 +5970,39 @@
 - Return an item to service, restoring it to availability checks</t>
         </is>
       </c>
-      <c r="G46" s="2" t="n">
+      <c r="G47" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>B-04</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr"/>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr"/>
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>E07 Equipment &amp; Technical Support</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>E07-S06</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>Request technical support for an event</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to request on-site technical support for an event and describe what is needed so that suitable staff can be allocated.</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Support request recorded
 Given an event requires technical support When I submit a request describing the support and the times it is needed Then the Technical Support Staff are notified and the request is recorded against the event
@@ -5849,39 +6018,39 @@
 - Mark an event as requiring no technical support</t>
         </is>
       </c>
-      <c r="G47" s="2" t="n">
+      <c r="G48" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>C-22, T-23</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr"/>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr"/>
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>E07 Equipment &amp; Technical Support</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>E07-S07</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>Assign and manage technical staff for an event</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>As a Technical Support Staff member, I want to assign and manage available colleagues to support an event so that the right people are on site at the right time.</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Available colleague assigned
 Given an event has an open technical support request and a colleague is available for its times When I assign them Then they are notified and the assignment appears on their schedule
@@ -5900,39 +6069,39 @@
 - Confirm the staff member is notified when assigned or removed</t>
         </is>
       </c>
-      <c r="G48" s="2" t="n">
+      <c r="G49" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>C-39</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr"/>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr"/>
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>E08 Readiness &amp; Confirmation</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>E08-S01</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>View readiness of an event</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to see whether venue, equipment and technical support are ready so that I know what still needs my attention.</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Arrangement states shown
 Given an event is in planning When I open its readiness view Then each arrangement is shown as complete, in progress or not started
@@ -5940,39 +6109,39 @@
 Given an arrangement is not started When I view it Then the responsible role and the action required are shown</t>
         </is>
       </c>
-      <c r="G49" s="2" t="n">
+      <c r="G50" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr"/>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr"/>
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>E08 Readiness &amp; Confirmation</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>E08-S02</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>Track outstanding actions across events</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want a list of upcoming events with incomplete arrangements so that nothing is overlooked before an event takes place.</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Incomplete events listed by date
 Given I have upcoming events with incomplete arrangements When I open my outstanding actions list Then those events are listed with the specific incomplete items, ordered by event date
@@ -5980,40 +6149,40 @@
 Given an event is close to its date and arrangements are still incomplete When I view the list Then that event is highlighted as urgent</t>
         </is>
       </c>
-      <c r="G50" s="2" t="n">
+      <c r="G51" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>C-28</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr"/>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="I51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr"/>
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>E08 Readiness &amp; Confirmation</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>E08-S03</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>Confirm an event</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to confirm an event once the event's arrangements are complete so that the Event Organiser and Attendees can rely on the details.
 Amended in place for the Week 7 Customer Changes (C-70, T-71; this story is To Do, T-74). Completing the arrangements no longer sets Confirmed directly: it lets the Coordinator submit the event for its Operational Safety Check, which moves it to the new Safety Review status, and the Safety Officer's approval (E08-S06) is what sets Confirmed. The readiness checks below are unchanged in substance; what they now gate is the submission. Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - All arrangements complete, event submitted for safety review
 Given every venue booking on the event is Confirmed or has been withdrawn, at least one is Confirmed, its full requested equipment is reserved and any requested technical support is assigned When I submit the event for its Operational Safety Check Then the status becomes Safety Review, the Safety Officer is notified, the Organiser is told the event is awaiting its safety check, and the event becomes Confirmed only when the Safety Officer approves it (E08-S06) (C-67, T-68, C-70, T-71; assumes O-28, O-39, O-40)
@@ -6039,39 +6208,39 @@
 - Confirm the Event Organiser is notified with the full confirmed details</t>
         </is>
       </c>
-      <c r="G51" s="2" t="n">
+      <c r="G52" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>C-13, C-39, C-59, C-63, T-02, T-24, T-27, C-67, T-68, O-28, C-70, T-71, T-74, O-39, O-40</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr"/>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="I52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr"/>
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>E08 Readiness &amp; Confirmation</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>E08-S04</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>Revert a confirmed event to planning</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to return a confirmed event to planning when an arrangement breaks so that its status reflects reality.</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Reverted with a recorded reason
 Given an event is Confirmed When I revert it to Planning and record a reason Then the status becomes Planning and the Event Organiser is notified with the reason
@@ -6090,39 +6259,39 @@
 - Confirm a reverted event must pass the Operational Safety Check again before it is Confirmed again</t>
         </is>
       </c>
-      <c r="G52" s="2" t="n">
+      <c r="G53" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>C-48, T-03, T-28, C-70, T-71</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr"/>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="I53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr"/>
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>E08 Readiness &amp; Confirmation</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>E08-S05</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>Complete an event</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want an event to become Completed once it has taken place so that attendance can be recorded and the event closed.</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Auto-completed after the end time
 Given an event is Confirmed and its end time has passed When the system next evaluates it Then the status becomes Completed
@@ -6140,40 +6309,40 @@
 - Confirm the transition is recorded in the activity log</t>
         </is>
       </c>
-      <c r="G53" s="2" t="n">
+      <c r="G54" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H53" s="2" t="inlineStr">
+      <c r="H54" s="2" t="inlineStr">
         <is>
           <t>T-03, T-26, T-48</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr"/>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="I54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr"/>
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>E08 Readiness &amp; Confirmation</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>E08-S06</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>Conduct the Operational Safety Check as the Safety Officer</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>As a Safety Officer, I want to review the operational safety of each event whose venue and technical arrangements are confirmed, and approve it, reject its safety arrangement or request changes, so that no event proceeds to preparation until it is safe to run.
 New story from the Week 7 Customer Changes (C-70) and the seventh role (T-72). The Safety Review status it works on sits between Planning and Confirmed as an interim placement (T-71); O-39 asks the customer to confirm. The customer guarantees a response, so there is no timeout path. Estimate at Sprint 3 planning (T-73). Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Events awaiting review listed with what the check needs
 Given events are in Safety Review When I open my queue Then each shows the event name, date and time, every confirmed venue with its capacity, layout and known restrictions, expected attendance, accessibility requirements, equipment and its placement, and the time it entered Safety Review, oldest first
@@ -6206,37 +6375,37 @@
 - Confirm every decision is in the activity log</t>
         </is>
       </c>
-      <c r="G54" s="2" t="inlineStr"/>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t>C-70, T-71, T-72, T-73, T-74, O-39, O-40, O-41, O-42, O-43</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr"/>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="I55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr"/>
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>E09 Attendee Registration</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>E09-S01</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>Register for an event</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>As an Attendee, I want to register for a confirmed event so that my place is reserved and I receive the event information.</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Place reserved in an open event
 Given an event is Confirmed, registration is open and places remain When I submit the required registration information Then my place is reserved and I receive a confirmation containing the event details
@@ -6257,39 +6426,39 @@
 - Be refused registration for an event that is not Confirmed</t>
         </is>
       </c>
-      <c r="G55" s="2" t="n">
+      <c r="G56" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H55" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>C-35, T-48, C-67, T-68, O-30</t>
         </is>
       </c>
-      <c r="I55" s="2" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr"/>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="I56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr"/>
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>E09 Attendee Registration</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>E09-S02</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>Enforce registration capacity</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>As an Event Organiser, I want registration to stop at the booked venue's capacity so that more people do not register than the venue can hold.</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Venue capacity enforced
 Given the event's capacity is the booked venue's capacity When registrations reach that number Then further registrations are refused
@@ -6310,39 +6479,39 @@
 - Confirm a manual addition is distinguishable from a normal registration</t>
         </is>
       </c>
-      <c r="G56" s="2" t="n">
+      <c r="G57" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="H57" s="2" t="inlineStr">
         <is>
           <t>C-05, C-58, T-30, T-31, T-50, B-11</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr"/>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="I57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr"/>
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>E09 Attendee Registration</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>E09-S03</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>Control the registration period</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>As an Event Organiser, I want to set when registration opens and closes, and when withdrawal closes, so that Attendees can act only during the permitted windows.</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Before registration opens
 Given the registration opening date has not been reached When an Attendee views the event Then registration is shown as not yet open and the opening date is stated
@@ -6361,39 +6530,39 @@
 - Be warned when setting a closing date after the event has started</t>
         </is>
       </c>
-      <c r="G57" s="2" t="n">
+      <c r="G58" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H57" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>C-24, C-44, T-42</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr"/>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="I58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr"/>
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>E09 Attendee Registration</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>E09-S04</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Join the waiting list</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>As an Attendee, I want to join the waiting list when an event is full so that I can still attend if a place is released.</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Joined a full event's list
 Given an event is full and the waiting list is enabled When I join the waiting list Then I am added and told I will be notified when a place is released
@@ -6412,39 +6581,39 @@
 - Confirm no waiting list is offered when the Organiser has disabled it</t>
         </is>
       </c>
-      <c r="G58" s="2" t="n">
+      <c r="G59" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>C-23, T-33, T-46, B-10</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr"/>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="I59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr"/>
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>E09 Attendee Registration</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>E09-S05</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>Withdraw my registration</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>As an Attendee, I want to withdraw my registration so that my place is released to someone else.</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Registration withdrawn
 Given I am registered and the withdrawal deadline has not passed When I withdraw Then my registration is cancelled and the place becomes available again
@@ -6456,39 +6625,39 @@
 - Be refused after the withdrawal deadline, with a contact provided</t>
         </is>
       </c>
-      <c r="G59" s="2" t="n">
+      <c r="G60" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>C-24, T-48, B-10</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr"/>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr"/>
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>E09 Attendee Registration</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>E09-S06</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>Record attendance</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to record which registered Attendees actually attended the event so that registration and attendance can be distinguished.</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Attendance marked after completion
 Given an event has status Completed When I mark an Attendee as attended for an event Then their record shows attended and the registration figure is unchanged
@@ -6504,39 +6673,39 @@
 - View registration and attendance counts side by side for the event</t>
         </is>
       </c>
-      <c r="G60" s="2" t="n">
+      <c r="G61" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t>C-45</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr"/>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="I61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr"/>
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>E09 Attendee Registration</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>E09-S07</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>View registrations for my event</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>As an Event Organiser, I want to view the list of Attendees registered for my event so that I can plan for the numbers attending the event.</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Registrations grouped by event
 Given Attendees have registered for my event When I open its registration list Then I see each Attendee's name, email address and contact number
@@ -6554,39 +6723,39 @@
 - Be refused access to registration lists for events I do not manage</t>
         </is>
       </c>
-      <c r="G61" s="2" t="n">
+      <c r="G62" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>C-26, T-32, O-05</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr"/>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="I62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr"/>
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>E10 Changes, Rescheduling &amp; Cancellation</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>E10-S01</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>Request a change after submission</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>As an Event Organiser, I want to request a change to my event after it has been submitted or confirmed so that the arrangements reflect what I now need.</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Change request recorded
 Given my event has been approved or confirmed When I submit a change request describing what should change Then the assigned Coordinator is notified and the request is recorded against the event
@@ -6605,39 +6774,39 @@
 - Be notified when the Coordinator approves or declines the request</t>
         </is>
       </c>
-      <c r="G62" s="2" t="n">
+      <c r="G63" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t>C-14, C-52, C-54, T-16</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr"/>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="I63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr"/>
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>E10 Changes, Rescheduling &amp; Cancellation</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>E10-S02</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>Distinguish minor edits from arrangement-affecting changes</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want the system to tell me when a change affects arrangements already confirmed so that I re-check them rather than assuming they still hold.</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Attendance beyond capacity flagged
 Given an event has one or more confirmed venue bookings When its expected attendance is increased Then each venue booking whose governing headcount (the booking's own headcount where set, otherwise the event's attendance) now exceeds that venue's capacity is flagged for review, and the others are not (C-67; assumes O-27) and the Venue Staff are notified
@@ -6658,39 +6827,39 @@
 - Confirm affected Venue Staff and Technical Support Staff are notified</t>
         </is>
       </c>
-      <c r="G63" s="2" t="n">
+      <c r="G64" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>C-05, T-16, B-05, B-11, C-67, T-68, O-27</t>
         </is>
       </c>
-      <c r="I63" s="2" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr"/>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr"/>
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>E10 Changes, Rescheduling &amp; Cancellation</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>E10-S03</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>Reschedule an event</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to reschedule an event to new dates so that it can still take place when the original dates no longer work.</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Date change flags bookings
 Given an event has a confirmed venue and equipment When I change its date Then the existing bookings are flagged as requiring reconfirmation and are not moved silently
@@ -6698,39 +6867,39 @@
 Given Attendees have registered for the event When it is rescheduled Then all registered Attendees are notified of the new date and time</t>
         </is>
       </c>
-      <c r="G64" s="2" t="n">
+      <c r="G65" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>C-25, O-18</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr"/>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="I65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr"/>
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>E10 Changes, Rescheduling &amp; Cancellation</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>E10-S04</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>Cancel an event</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to cancel an event and release its arrangements so that venues and equipment do not stay committed to something that will not happen.</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Event cancelled, arrangements released
 Given an Event Organiser requests cancellation When I cancel the event and record a reason Then its status becomes Cancelled, its venue booking and equipment reservations are released, the venue calendar is updated and the affected staff are notified
@@ -6749,52 +6918,12 @@
 - Confirm a cancelled event is read-only and shows its reason and date</t>
         </is>
       </c>
-      <c r="G65" s="2" t="n">
+      <c r="G66" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>C-14, C-54, T-07, T-48</t>
-        </is>
-      </c>
-      <c r="I65" s="2" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr"/>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>E10 Changes, Rescheduling &amp; Cancellation</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>E10-S05</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>Handle a venue lost from a confirmed event</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>As an Event Coordinator, I want to be alerted when a venue becomes unavailable for one of my confirmed events so that I can arrange an alternative before Attendees are affected.</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="inlineStr">
-        <is>
-          <t>Scenario 1 - Blocked venue flags the event
-Given my event has a confirmed venue When Venue Staff block that venue over the event's period Then I am notified and the event is flagged as at risk
-Scenario 2 - At-risk event offers a new search
-Given my event is flagged as at risk When I open it Then the reason and the affected arrangement are shown and I can begin a new venue search from that screen</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr"/>
@@ -6803,25 +6932,76 @@
       <c r="A67" s="2" t="inlineStr"/>
       <c r="B67" s="2" t="inlineStr">
         <is>
+          <t>E10 Changes, Rescheduling &amp; Cancellation</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>E10-S05</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Handle a venue lost from a confirmed event</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>As an Event Coordinator, I want to be alerted when a venue becomes unavailable for one of my events and to find and request a replacement from the event itself, so that I can arrange an alternative before Attendees are affected while the original event information is preserved.
+Returned to Release 1 by the Week 7 Customer Changes (C-66, T-67). The three-point estimate is carried from the original backlog and re-estimated at Sprint 3 planning (T-73). The alert itself is raised by E05-S06; this story is what the Coordinator does with it. Scenarios tagged "(assumes O-xx)" are written to the default recorded in `docs/bdr/C-open-questions.md`.</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Scenario 1 - Lost venue flags the event
+Given my event has a Pending or Confirmed venue booking When Venue Staff mark that venue unavailable over the booking's period (E05-S06) Then I am notified, the booking shows as Conflicting on the event, and the event is flagged as needing alternative arrangements while its status and every other arrangement stay as they were (assumes O-24)
+Scenario 2 - Flagged event offers a replacement search
+Given my event is flagged When I open it Then the reason category, the period and the affected booking are shown, the original venue, dates and requirements are preserved, and I can start a venue search (E06-S01) for the same event from that screen
+Scenario 3 - Replacement requested without losing the original
+Given I have found a replacement venue When I submit a booking request for it (E06-S03) Then the request is created for the same event alongside the Conflicting booking, and I may cancel the Conflicting booking explicitly once the replacement is Confirmed; nothing is cancelled for me
+Scenario 4 - Organiser and Attendees told on the actual change
+Given I confirm a replacement venue When the venue of a Confirmed event changes Then the Organiser and registered Attendees are notified of the new venue through the existing venue-change routing (E11-S01), and not earlier (assumes O-25)
+Checklist
+- Be notified when a venue I have booked is marked unavailable over my booking
+- See the reason, period and affected booking on the event, with the original event information intact
+- Start a venue search for the same event from the flagged event
+- Request a replacement venue while the Conflicting booking remains on the event until I cancel it
+- Confirm the Organiser and registered Attendees are told of the venue change only when it actually happens</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>C-66, C-61, T-28, T-67, T-73, T-74, O-24, O-25</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr"/>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
           <t>E11 Notifications &amp; Reminders</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
         <is>
           <t>E11-S01</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>Notify users about events they are involved in</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>As a user involved in an event, I want to be notified when its status or arrangements change so that I do not have to keep checking the system and nobody continues working from outdated information.</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Status change notified
 Given I am a recipient under the approved routing matrix When an event status changes or a booking decision is made Then I receive a notification stating what changed, when, and which event it concerns, unless I performed the action myself
@@ -6849,39 +7029,39 @@
 - Mark a notification as read</t>
         </is>
       </c>
-      <c r="G67" s="2" t="n">
+      <c r="G68" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="H68" s="2" t="inlineStr">
         <is>
           <t>C-04, C-29, C-53, T-35, T-36, T-44, T-48, T-64, C-68, T-69, O-33, C-69, T-70, C-70, T-71</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr"/>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="I68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr"/>
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>E11 Notifications &amp; Reminders</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>E11-S03</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>Receive reminders about upcoming commitments</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>As a Technical Support Staff member, I want reminders about upcoming events I am supporting so that equipment and support are prepared in time.</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Reminder lists requirements
 Given I am assigned to an upcoming event When the reminder point before it is reached Then I receive a reminder listing the equipment and support required
@@ -6889,39 +7069,39 @@
 Given an event is cancelled before its reminder is due When the reminder point is reached Then no reminder is sent</t>
         </is>
       </c>
-      <c r="G68" s="2" t="n">
+      <c r="G69" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>C-28, O-11</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr"/>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="I69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr"/>
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>E11 Notifications &amp; Reminders</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>E11-S04</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>Alert on incomplete arrangements</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to be alerted when an upcoming event still has incomplete arrangements so that I can act while there is still time.</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Incomplete items named
 Given an upcoming event has an incomplete essential arrangement When the alert point before it is reached Then I receive an alert naming the incomplete items
@@ -6929,39 +7109,39 @@
 Given all arrangements are completed before the alert point When the alert point is reached Then no alert is sent</t>
         </is>
       </c>
-      <c r="G69" s="2" t="n">
+      <c r="G70" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr"/>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="I70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr"/>
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>E12 Calendar, Search &amp; Dashboards</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>E12-S01</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>View my events in a calendar</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to see my events in a calendar so that I can plan my workload across the coming weeks.</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr">
+      <c r="F71" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Events shown on their dates
 Given I have events spread across several weeks When I open the calendar Then my events appear on their dates with their status indicated
@@ -6969,39 +7149,39 @@
 Given an event spans several days When I view the calendar Then it is shown across all its days rather than only the first</t>
         </is>
       </c>
-      <c r="G70" s="2" t="n">
+      <c r="G71" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H70" s="2" t="inlineStr">
+      <c r="H71" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr"/>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="I71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr"/>
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>E12 Calendar, Search &amp; Dashboards</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>E12-S02</t>
         </is>
       </c>
-      <c r="D71" s="2" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr">
         <is>
           <t>Search and filter events</t>
         </is>
       </c>
-      <c r="E71" s="2" t="inlineStr">
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to search events by name, client, date, venue, status, category or assigned Coordinator so that I can find a specific event quickly.</t>
         </is>
       </c>
-      <c r="F71" s="2" t="inlineStr">
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Permitted matches returned
 Given events match my criteria When I search Then only matching events that I am permitted to see are returned
@@ -7011,39 +7191,39 @@
 Given I apply several filters at once When I search Then all the filters are applied together</t>
         </is>
       </c>
-      <c r="G71" s="2" t="n">
+      <c r="G72" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H71" s="2" t="inlineStr">
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr"/>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="I72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr"/>
+      <c r="B73" s="2" t="inlineStr">
         <is>
           <t>E12 Calendar, Search &amp; Dashboards</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>E12-S03</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr">
         <is>
           <t>See my work on a role-based dashboard</t>
         </is>
       </c>
-      <c r="E72" s="2" t="inlineStr">
+      <c r="E73" s="2" t="inlineStr">
         <is>
           <t>As a Venue Staff member, I want a dashboard showing booking requests awaiting my decision and upcoming venue preparations so that I can see my outstanding work in one place.</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr">
+      <c r="F73" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Pending decisions listed
 Given booking requests are pending my decision When I open my dashboard Then they are listed with event name, venue, dates and how long each has been waiting
@@ -7051,39 +7231,39 @@
 Given I have no outstanding items When I open my dashboard Then an empty state is shown rather than an error</t>
         </is>
       </c>
-      <c r="G72" s="2" t="n">
+      <c r="G73" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H72" s="2" t="inlineStr">
+      <c r="H73" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I72" s="2" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr"/>
-      <c r="B73" s="2" t="inlineStr">
+      <c r="I73" s="2" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr"/>
+      <c r="B74" s="2" t="inlineStr">
         <is>
           <t>E12 Calendar, Search &amp; Dashboards</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr">
+      <c r="C74" s="2" t="inlineStr">
         <is>
           <t>E12-S04</t>
         </is>
       </c>
-      <c r="D73" s="2" t="inlineStr">
+      <c r="D74" s="2" t="inlineStr">
         <is>
           <t>Use the system on a mobile device</t>
         </is>
       </c>
-      <c r="E73" s="2" t="inlineStr">
+      <c r="E74" s="2" t="inlineStr">
         <is>
           <t>As a Venue Staff member, I want to use the system on my phone while preparing a venue so that I can check and update arrangements without returning to a desk.</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr">
+      <c r="F74" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Readable without horizontal scrolling
 Given I open the system on a mobile device When I view my dashboard, an event or a venue calendar Then the content is readable and usable without horizontal scrolling
@@ -7091,39 +7271,39 @@
 Given I am working on a mobile device When I update a preparation status Then the update is saved exactly as it would be on a desktop</t>
         </is>
       </c>
-      <c r="G73" s="2" t="n">
+      <c r="G74" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H73" s="2" t="inlineStr">
+      <c r="H74" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I73" s="2" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr"/>
-      <c r="B74" s="2" t="inlineStr">
+      <c r="I74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr"/>
+      <c r="B75" s="2" t="inlineStr">
         <is>
           <t>E13 Reporting &amp; Export</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
+      <c r="C75" s="2" t="inlineStr">
         <is>
           <t>E13-S01</t>
         </is>
       </c>
-      <c r="D74" s="2" t="inlineStr">
+      <c r="D75" s="2" t="inlineStr">
         <is>
           <t>Generate an event report</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr">
+      <c r="E75" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to generate a summary report for an event so that I can share the arrangements at operational meetings.</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr">
+      <c r="F75" s="2" t="inlineStr">
         <is>
           <t>Checklist
 - Generate a downloadable report containing event name, date and time, venue, equipment list, assigned technical support and total registered Attendees
@@ -7132,39 +7312,39 @@
 - Show a clear error with a retry option if generation fails</t>
         </is>
       </c>
-      <c r="G74" s="2" t="n">
+      <c r="G75" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H74" s="2" t="inlineStr">
+      <c r="H75" s="2" t="inlineStr">
         <is>
           <t>C-27, O-01</t>
         </is>
       </c>
-      <c r="I74" s="2" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr"/>
-      <c r="B75" s="2" t="inlineStr">
+      <c r="I75" s="2" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr"/>
+      <c r="B76" s="2" t="inlineStr">
         <is>
           <t>E13 Reporting &amp; Export</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr">
+      <c r="C76" s="2" t="inlineStr">
         <is>
           <t>E13-S02</t>
         </is>
       </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="D76" s="2" t="inlineStr">
         <is>
           <t>Review venue usage over a period</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr">
+      <c r="E76" s="2" t="inlineStr">
         <is>
           <t>As a Venue Staff member, I want to review venue bookings and usage over a chosen period so that I can plan maintenance and identify under-used spaces.</t>
         </is>
       </c>
-      <c r="F75" s="2" t="inlineStr">
+      <c r="F76" s="2" t="inlineStr">
         <is>
           <t>Checklist
 - Select a custom date range with start and end dates
@@ -7174,39 +7354,39 @@
 - See an informative empty state when no records match</t>
         </is>
       </c>
-      <c r="G75" s="2" t="n">
+      <c r="G76" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="H75" s="2" t="inlineStr">
+      <c r="H76" s="2" t="inlineStr">
         <is>
           <t>C-27, O-01</t>
         </is>
       </c>
-      <c r="I75" s="2" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr"/>
-      <c r="B76" s="2" t="inlineStr">
+      <c r="I76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr"/>
+      <c r="B77" s="2" t="inlineStr">
         <is>
           <t>E13 Reporting &amp; Export</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr">
+      <c r="C77" s="2" t="inlineStr">
         <is>
           <t>E13-S03</t>
         </is>
       </c>
-      <c r="D76" s="2" t="inlineStr">
+      <c r="D77" s="2" t="inlineStr">
         <is>
           <t>Export attendee registration information</t>
         </is>
       </c>
-      <c r="E76" s="2" t="inlineStr">
+      <c r="E77" s="2" t="inlineStr">
         <is>
           <t>As an Event Organiser, I want to export the registration list for my event so that I can prepare badges and catering numbers.</t>
         </is>
       </c>
-      <c r="F76" s="2" t="inlineStr">
+      <c r="F77" s="2" t="inlineStr">
         <is>
           <t>Checklist
 - Export registrations only for events the Organiser manages
@@ -7214,39 +7394,39 @@
 - Exclude sensitive personal data from the generated file</t>
         </is>
       </c>
-      <c r="G76" s="2" t="n">
+      <c r="G77" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H76" s="2" t="inlineStr">
+      <c r="H77" s="2" t="inlineStr">
         <is>
           <t>C-26, T-32</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr"/>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="I77" s="2" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr"/>
+      <c r="B78" s="2" t="inlineStr">
         <is>
           <t>E14 Audit &amp; History</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="C78" s="2" t="inlineStr">
         <is>
           <t>E14-S01</t>
         </is>
       </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="D78" s="2" t="inlineStr">
         <is>
           <t>View an event's change history</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr">
+      <c r="E78" s="2" t="inlineStr">
         <is>
           <t>As an Event Coordinator, I want to see how an event's important information has changed over time so that I can explain how the current arrangements were reached.</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr">
+      <c r="F78" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Before and after values listed
 Given an event's date, venue, attendance or status has changed When I open its change history Then each change is listed with the previous value, the new value, who made it and when
@@ -7254,39 +7434,39 @@
 Given I am not permitted to view a particular change When I open the history Then that entry is not shown to me</t>
         </is>
       </c>
-      <c r="G77" s="2" t="n">
+      <c r="G78" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H77" s="2" t="inlineStr">
+      <c r="H78" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I77" s="2" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr"/>
-      <c r="B78" s="2" t="inlineStr">
+      <c r="I78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr"/>
+      <c r="B79" s="2" t="inlineStr">
         <is>
           <t>E14 Audit &amp; History</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="C79" s="2" t="inlineStr">
         <is>
           <t>E14-S02</t>
         </is>
       </c>
-      <c r="D78" s="2" t="inlineStr">
+      <c r="D79" s="2" t="inlineStr">
         <is>
           <t>Record significant actions in an activity log</t>
         </is>
       </c>
-      <c r="E78" s="2" t="inlineStr">
+      <c r="E79" s="2" t="inlineStr">
         <is>
           <t>As a ConnectSphere staff member, I want significant actions to be recorded so that we can determine who did what and when.</t>
         </is>
       </c>
-      <c r="F78" s="2" t="inlineStr">
+      <c r="F79" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Status change recorded
 Given an event status changes When the change completes Then an entry is recorded with the actor, the action, the affected event and the time
@@ -7306,15 +7486,15 @@
 - Confirm log entries cannot be edited or deleted by any user</t>
         </is>
       </c>
-      <c r="G78" s="2" t="n">
+      <c r="G79" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H78" s="2" t="inlineStr">
+      <c r="H79" s="2" t="inlineStr">
         <is>
           <t>T-04</t>
         </is>
       </c>
-      <c r="I78" s="2" t="inlineStr"/>
+      <c r="I79" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>